<commit_message>
Rediseña la página: Navidad, saludo editable, año automático y otros calendarios
- Agrega más ciudades grandes a países que solo mostraban una secundaria
  (Beijing, Dubái, Mumbai, San Petersburgo, Karachi, etc.)
- Reordena las zonas de UTC+14 a UTC-12
- Cambia el acento amarillo por un verde azulado, y ensancha el layout
  para aprovechar mejor el espacio (grilla de zonas en columnas)
- Los tuits ahora se arman en el navegador a partir de data.json + un
  saludo editable (persistido en localStorage), así el año se actualiza
  solo cada temporada sin tocar el código
- Agrega una pestaña "Navidad" (mismas ciudades, saludo y fecha propios)
  y otra de "Otros calendarios" con las fechas exactas de Rosh Hashaná,
  Año Nuevo chino, Nowruz, Enkutatash, Songkran y el Año Nuevo islámico

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ciudades_Uso_Horario_2027_CORREGIDO.xlsx
+++ b/Ciudades_Uso_Horario_2027_CORREGIDO.xlsx
@@ -644,7 +644,7 @@
           <t>🇨🇦 Vancouver / Dawson - Canada (Canada)
 🇫🇷 Île Clipperton - France (Clipperton Island - France)
 🇵🇳 Adamstown - Pitcairn Islands (Pitcairn Island)
-🇺🇸 Los Angeles / Seattle - United States (USA)</t>
+🇺🇸 Los Angeles / San Francisco / Seattle - United States (USA)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -714,9 +714,9 @@
 🇸🇻 San Salvador - El Salvador (El Salvador)
 🇬🇹 Ciudad de Guatemala - Guatemala (Guatemala)
 🇭🇳 Tegucigalpa - Honduras (Honduras)
-🇲🇽 Ciudad de México - México (Mexico)
+🇲🇽 Ciudad de México / Guadalajara / Monterrey - México (Mexico)
 🇳🇮 Managua - Nicaragua (Nicaragua)
-🇺🇸 Dallas - United States (USA)</t>
+🇺🇸 Chicago / Dallas - United States (USA)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -886,7 +886,7 @@
           <t>🇦🇶 Rothera Research Station - Antarctica / United Kingdom (Antarctica / UK)
 🇦🇶 Palmer Station - Antarctica / United States (Antarctica / USA)
 🇦🇶 Base Marambio - Antártida / Argentina (Antarctica / Argentina)
-🇦🇷 Buenos Aires - Argentina (Argentina)
+🇦🇷 Buenos Aires / Córdoba / Rosario - Argentina (Argentina)
 🇦🇷 Islas Georgias del Sur - Argentina (South Georgia Islands)
 🇦🇷 Islas Sandwich del Sur - Argentina (South Sandwich Islands)
 🇦🇷 Puerto Argentino - Argentina
@@ -1063,16 +1063,16 @@
 🇨🇬 Brazzaville - Congo (Congo)
 🇲🇪 Podgorica - Crna Gora (Montenegro)
 🇩🇰 København (Copenhagen) - Danmark (Denmark)
-🇩🇪 Berlin - Deutschland (Germany)
+🇩🇪 Berlin / Hamburg / München (Munich) - Deutschland (Germany)
 🇪🇸 Ceuta - España (Spain)
-🇪🇸 Madrid - España (Spain)
+🇪🇸 Madrid / Barcelona - España (Spain)
 🇪🇸 Melilla - España (Spain)
-🇫🇷 Paris - France (France)
+🇫🇷 Paris / Marseille / Lyon - France (France)
 🇬🇦 Libreville - Gabon (Gabon)
 🇬🇮 Gibraltar - Gibraltar (Gibraltar - UK)
 🇬🇶 Malabo - Guinea Ecuatorial (Equatorial Guinea)
 🇭🇷 Zagreb - Hrvatska (Croatia)
-🇮🇹 Roma (Rome) - Italia (Italy)
+🇮🇹 Roma (Rome) / Milano (Milan) - Italia (Italy)
 🇽🇰 Prishtinë (Pristina) - Kosova (Kosovo)
 🇱🇮 Vaduz - Liechtenstein (Liechtenstein)
 🇱🇺 Luxembourg - Luxembourg (Luxembourg)
@@ -1115,7 +1115,7 @@
         <v>47</v>
       </c>
       <c r="G17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
@@ -1199,11 +1199,11 @@
 🇹🇷 Ankara / İstanbul / Lefkoşa (Kuzey Kıbrıs) - Türkiye (Turkey / Northern Cyprus)
 🇺🇬 Kampala - Uganda (Uganda)
 🇧🇾 Мінск (Minsk) - Беларусь (Belarus)
-🇷🇺 Москва (Moscow) - Россия (Russia)
+🇷🇺 Москва (Moscow) / Санкт-Петербург (Saint Petersburg) - Россия (Russia)
 🇯🇴 عمان (Amman) - الأردن (Jordan)
 🇧🇭 المنامة (Manama) - البحرين (Bahrain)
 🇮🇶 بغداد (Baghdad) - العراق (Iraq)
-🇸🇦 الرياض (Riyadh) - العربية السعودية (Saudi Arabia)
+🇸🇦 الرياض (Riyadh) / جدة (Jeddah) - العربية السعودية (Saudi Arabia)
 🇰🇼 مدينة الكويت (Kuwait City) - الكويت (Kuwait)
 🇾🇪 صنعاء (Sana'a) - اليمن (Yemen)
 🇸🇾 دمشق (Damascus) - سوريا (Syria)
@@ -1277,7 +1277,7 @@
 🇸🇨 Victoria - Seychelles (Seychelles)
 🇷🇺 Самара (Samara) - Россия (Russia)
 🇦🇲 Երևան (Yerevan) - Հայաստան (Armenia)
-🇦🇪 أبو ظبي (Abu Dhabi) - الإمارات العربية المتحدة (UAE)
+🇦🇪 أبو ظبي (Abu Dhabi) / دبي (Dubai) - الإمارات العربية المتحدة (UAE)
 🇴🇲 مَسْقَط (Muscat) - عُمان (Oman)
 🇬🇪 თბილისი (Tbilisi) - საქართველო (Georgia)</t>
         </is>
@@ -1347,7 +1347,7 @@
 🇷🇺 Екатеринбург (Yekaterinburg) - Россия (Russia)
 🇹🇯 Душанбе (Dushanbe) - Тоҷикистон (Tajikistan)
 🇰🇿 Астана / Алматы (Astana / Almaty) - Қазақстан (Kazakhstan)
-🇵🇰 اسلام آباد (Islamabad) - پاکستان (Pakistan)
+🇵🇰 اسلام آباد (Islamabad) / کراچی (Karachi) - پاکستان (Pakistan)
 🇲🇻 မާލެ (Malé) - ދިވެހިރާއްޖެ (Maldives)</t>
         </is>
       </c>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>🇮🇳 नई दिल्ली (New Delhi) - भारत (India)
+          <t>🇮🇳 नई दिल्ली (New Delhi) / मुंबई (Mumbai) / बेंगलुरु (Bangalore) - भारत (India)
 🇱🇰 ශ්‍රီ ජයවර්ධනපුර කෝට්ටེ་ (Sri Jayawardenepura Kotte) - ශ්‍රီ ලංකා (Sri Lanka)</t>
         </is>
       </c>
@@ -1512,7 +1512,7 @@
           <t>🇦🇶 Davis Station - Antarctica / Australia (Antarctica / Australia)
 🇨🇽 Flying Fish Cove - Christmas Island (Christmas Island)
 🇮🇩 Jakarta - Indonesia (Indonesia)
-🇻🇳 Hà Nội (Hanoi) - Việt Nam (Vietnam)
+🇻🇳 Hà Nội (Hanoi) / Thành phố Hồ Chí Minh (Ho Chi Minh City) - Việt Nam (Vietnam)
 🇲🇳 Ховд (Hovd) - Монгол Улс (Mongolia)
 🇷🇺 Красноярск / Новосибирск (Krasnoyarsk / Novosibirsk) - Россия (Russia)
 🇹🇭 กรุงเทพมหานคร (Bangkok) - ประเทศไทย (Thailand)
@@ -1556,7 +1556,7 @@
 🇸🇬 Singapore / 新加坡 / சிங்கப்பூர் - Singapore (Singapore)
 🇲🇳 Улаанбаатар / Хархорум (Ulaanbaatar / Kharkhorum) - Монгол Улс (Mongolia)
 🇷🇺 Иркутск (Irkutsk) - Россия (Russia)
-🇨🇳 上海 (Shanghai) - 中国 (China)
+🇨🇳 北京 (Beijing) / 上海 (Shanghai) - 中国 (China)
 🇹🇼 台北 (Taipei) - 台灣 (Taiwan)
 🇲🇴 澳門 (Macau) - 澳門 (Macau)
 🇭🇰 香港 (Hong Kong) - 香港 (Hong Kong)</t>
@@ -1594,9 +1594,9 @@
 🇮🇩 Jayapura - Indonesia (Indonesia)
 🇹🇱 Dili - Timor-Leste (Timor-Leste)
 🇷🇺 Якутск (Yakutsk) - Россия (Russia)
-🇰🇷 서울 (Seoul) - 대한민국 (South Korea)
+🇰🇷 서울 (Seoul) / 부산 (Busan) - 대한민국 (South Korea)
 🇰🇵 평양 (Pyongyang) - 조선민주주의인민공화국 (North Korea)
-🇯🇵 東京 (Tokyo) - 日本 (Japan)</t>
+🇯🇵 東京 (Tokyo) / 大阪 (Osaka) - 日本 (Japan)</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>239</v>
+        <v>255</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
@@ -2102,7 +2102,7 @@
 🇨🇦 Vancouver / Dawson - Canada (Canada)
 🇫🇷 Île Clipperton - France (Clipperton Island - France)
 🇵🇳 Adamstown - Pitcairn Islands (Pitcairn Island)
-🇺🇸 Los Angeles / Seattle - United States (USA)</t>
+🇺🇸 Los Angeles / San Francisco / Seattle - United States (USA)</t>
         </is>
       </c>
     </row>
@@ -2180,7 +2180,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>195</v>
+        <v>231</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -2188,9 +2188,9 @@
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC-6
 🇭🇳 Tegucigalpa - Honduras (Honduras)
-🇲🇽 Ciudad de México - México (Mexico)
+🇲🇽 Ciudad de México / Guadalajara / Monterrey - México (Mexico)
 🇳🇮 Managua - Nicaragua (Nicaragua)
-🇺🇸 Dallas - United States (USA)
+🇺🇸 Chicago / Dallas - United States (USA)
 (2/2)</t>
         </is>
       </c>
@@ -2570,14 +2570,14 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>250</v>
+        <v>270</v>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC-3
-🇦🇷 Buenos Aires - Argentina (Argentina)
+🇦🇷 Buenos Aires / Córdoba / Rosario - Argentina (Argentina)
 🇦🇷 Islas Georgias del Sur - Argentina (South Georgia Islands)
 🇦🇷 Islas Sandwich del Sur - Argentina (South Sandwich Islands)
 🇦🇷 Puerto Argentino - Argentina
@@ -2948,11 +2948,11 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1/9</t>
+          <t>1/10</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
@@ -2964,7 +2964,7 @@
 🇧🇪 Bruxelles / Brussel (Brussels) - Belgique / België (Belgium)
 🇧🇯 Porto-Novo - Bénin (Benin)
 🇧🇦 Sarajevo - Bosna i Hercegovina (Bosnia and Herzegovina)
-(1/9)</t>
+(1/10)</t>
         </is>
       </c>
     </row>
@@ -2979,11 +2979,11 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2/9</t>
+          <t>2/10</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
@@ -2995,7 +2995,7 @@
 🇻🇦 Città del Vaticano - Civitas Vaticana (Vatican City)
 🇨🇬 Brazzaville - Congo (Congo)
 🇲🇪 Podgorica - Crna Gora (Montenegro)
-(2/9)</t>
+(2/10)</t>
         </is>
       </c>
     </row>
@@ -3010,11 +3010,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3/9</t>
+          <t>3/10</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>271</v>
+        <v>256</v>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
@@ -3022,13 +3022,11 @@
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+1
 🇩🇰 København (Copenhagen) - Danmark (Denmark)
-🇩🇪 Berlin - Deutschland (Germany)
+🇩🇪 Berlin / Hamburg / München (Munich) - Deutschland (Germany)
 🇪🇸 Ceuta - España (Spain)
-🇪🇸 Madrid - España (Spain)
+🇪🇸 Madrid / Barcelona - España (Spain)
 🇪🇸 Melilla - España (Spain)
-🇫🇷 Paris - France (France)
-🇬🇦 Libreville - Gabon (Gabon)
-(3/9)</t>
+(3/10)</t>
         </is>
       </c>
     </row>
@@ -3043,23 +3041,23 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>4/9</t>
+          <t>4/10</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+1
+🇫🇷 Paris / Marseille / Lyon - France (France)
+🇬🇦 Libreville - Gabon (Gabon)
 🇬🇮 Gibraltar - Gibraltar (Gibraltar - UK)
 🇬🇶 Malabo - Guinea Ecuatorial (Equatorial Guinea)
 🇭🇷 Zagreb - Hrvatska (Croatia)
-🇮🇹 Roma (Rome) - Italia (Italy)
-🇽🇰 Prishtinë (Pristina) - Kosova (Kosovo)
-(4/9)</t>
+(4/10)</t>
         </is>
       </c>
     </row>
@@ -3074,55 +3072,55 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>5/9</t>
+          <t>5/10</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+1
+🇮🇹 Roma (Rome) / Milano (Milan) - Italia (Italy)
+🇽🇰 Prishtinë (Pristina) - Kosova (Kosovo)
 🇱🇮 Vaduz - Liechtenstein (Liechtenstein)
 🇱🇺 Luxembourg - Luxembourg (Luxembourg)
 🇭🇺 Budapest - Magyarország (Hungary)
+(5/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>UTC+1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>6/10</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>249</v>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
+🎇🥂🌟🪅💫💙🎉✨🍾🎆
+UTC+1
 🇲🇹 Valletta - Malta (Malta)
 🇳🇱 Amsterdam - Nederland (Netherlands)
 🇳🇪 Niamey - Niger (Niger)
-(5/9)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>1</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>UTC+1</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>6/9</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>259</v>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
-🎇🥂🌟🪅💫💙🎉✨🍾🎆
-UTC+1
 🇳🇬 Abuja / Lagos - Nigeria (Nigeria)
 🇳🇴 Oslo - Norge (Norway)
 🇦🇹 Wien (Vienna) - Österreich (Austria)
-🇵🇱 Warszawa (Warsaw) - Polska (Poland)
-🇲🇨 Monaco-Ville - Principauté de Monaco (Principality of Monaco)
-(6/9)</t>
+(6/10)</t>
         </is>
       </c>
     </row>
@@ -3137,105 +3135,133 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>7/9</t>
+          <t>7/10</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>268</v>
+        <v>223</v>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+1
+🇵🇱 Warszawa (Warsaw) - Polska (Poland)
+🇲🇨 Monaco-Ville - Principauté de Monaco (Principality of Monaco)
 🇨🇫 Bangui - République centrafricaine (Central African Republic)
+(7/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>UTC+1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>245</v>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
+🎇🥂🌟🪅💫💙🎉✨🍾🎆
+UTC+1
 🇨🇩 Kinshasa - République Démocratique du Congo (DR Congo)
 🇸🇲 San Marino - San Marino (San Marino)
 🇨🇭 Bern - Schweiz / Suisse / Svizzera (Switzerland)
-(7/9)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
+🇦🇱 Tiranë (Tirana) - Shqipëria (Albania)
+(8/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
         <v>1</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>UTC+1</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>8/9</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>227</v>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>9/10</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>245</v>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+1
-🇦🇱 Tiranë (Tirana) - Shqipëria (Albania)
 🇸🇮 Ljubljana - Slovenija (Slovenia)
 🇸🇰 Bratislava - Slovensko (Slovakia)
 🇸🇪 Stockholm - Sverige (Sweden)
 🇹🇩 N'Djaména - Tchad (Chad)
-(8/9)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
+🇲🇰 Скопје (Skopje) - Северна Македонија (North Macedonia)
+(9/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
         <v>1</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>UTC+1</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>9/9</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>253</v>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>10/10</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>197</v>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+1
-🇲🇰 Скопје (Skopje) - Северна Македонија (North Macedonia)
 🇷🇸 Београд (Belgrade) - Србија (Serbia)
 🇩🇿 الجزائر (Algiers) - الجزائر (Algeria)
 🇲🇦 Rabat - المغرب (Morocco)
 🇹🇳 تونس (Tunis) - تونس (Tunisia)
-(9/9)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
+(10/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
         <v>2</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>UTC+2</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>1/6</t>
         </is>
       </c>
-      <c r="D45" t="n">
+      <c r="D46" t="n">
         <v>262</v>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3250,24 +3276,24 @@
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="n">
+    <row r="47">
+      <c r="A47" t="n">
         <v>2</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>UTC+2</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>2/6</t>
         </is>
       </c>
-      <c r="D46" t="n">
+      <c r="D47" t="n">
         <v>246</v>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3282,24 +3308,24 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="n">
+    <row r="48">
+      <c r="A48" t="n">
         <v>2</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>UTC+2</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>3/6</t>
         </is>
       </c>
-      <c r="D47" t="n">
+      <c r="D48" t="n">
         <v>250</v>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3312,24 +3338,24 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="n">
+    <row r="49">
+      <c r="A49" t="n">
         <v>2</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>UTC+2</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>4/6</t>
         </is>
       </c>
-      <c r="D48" t="n">
+      <c r="D49" t="n">
         <v>266</v>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3344,24 +3370,24 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="n">
+    <row r="50">
+      <c r="A50" t="n">
         <v>2</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>UTC+2</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>5/6</t>
         </is>
       </c>
-      <c r="D49" t="n">
+      <c r="D50" t="n">
         <v>259</v>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3375,24 +3401,24 @@
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="n">
+    <row r="51">
+      <c r="A51" t="n">
         <v>2</v>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>UTC+2</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>6/6</t>
         </is>
       </c>
-      <c r="D50" t="n">
+      <c r="D51" t="n">
         <v>112</v>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3402,24 +3428,24 @@
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="n">
+    <row r="52">
+      <c r="A52" t="n">
         <v>3</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>UTC+3</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>1/5</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D52" t="n">
         <v>249</v>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3434,24 +3460,24 @@
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" t="n">
+    <row r="53">
+      <c r="A53" t="n">
         <v>3</v>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>UTC+3</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>2/5</t>
         </is>
       </c>
-      <c r="D52" t="n">
+      <c r="D53" t="n">
         <v>252</v>
       </c>
-      <c r="E52" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3464,115 +3490,115 @@
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" t="n">
+    <row r="54">
+      <c r="A54" t="n">
         <v>3</v>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>UTC+3</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>3/5</t>
         </is>
       </c>
-      <c r="D53" t="n">
-        <v>266</v>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="D54" t="n">
+        <v>268</v>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+3
 🇺🇬 Kampala - Uganda (Uganda)
 🇧🇾 Мінск (Minsk) - Беларусь (Belarus)
-🇷🇺 Москва (Moscow) - Россия (Russia)
+🇷🇺 Москва (Moscow) / Санкт-Петербург (Saint Petersburg) - Россия (Russia)
 🇯🇴 عمان (Amman) - الأردن (Jordan)
 🇧🇭 المنامة (Manama) - البحرين (Bahrain)
+(3/5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>3</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>UTC+3</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>4/5</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>273</v>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
+🎇🥂🌟🪅💫💙🎉✨🍾🎆
+UTC+3
 🇮🇶 بغداد (Baghdad) - العراق (Iraq)
-(3/5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>3</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>UTC+3</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>4/5</t>
-        </is>
-      </c>
-      <c r="D54" t="n">
-        <v>254</v>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
-🎇🥂🌟🪅💫💙🎉✨🍾🎆
-UTC+3
-🇸🇦 الرياض (Riyadh) - العربية السعودية (Saudi Arabia)
+🇸🇦 الرياض (Riyadh) / جدة (Jeddah) - العربية السعودية (Saudi Arabia)
 🇰🇼 مدينة الكويت (Kuwait City) - الكويت (Kuwait)
 🇾🇪 صنعاء (Sana'a) - اليمن (Yemen)
 🇸🇾 دمشق (Damascus) - سوريا (Syria)
+(4/5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>3</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>UTC+3</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>5/5</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>164</v>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
+🎇🥂🌟🪅💫💙🎉✨🍾🎆
+UTC+3
 🇶🇦 الدوحة (Doha) - قطر (Qatar)
-(4/5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>3</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>UTC+3</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>5/5</t>
-        </is>
-      </c>
-      <c r="D55" t="n">
-        <v>133</v>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
-🎇🥂🌟🪅💫💙🎉✨🍾🎆
-UTC+3
 🇱🇧 بيروت (Beirut) - لبنان (Lebanon)
 🇪🇹 အዲስ አበባ (Addis Ababa) - ኢትዮጵያ (Ethiopia)
 (5/5)</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" t="n">
+    <row r="57">
+      <c r="A57" t="n">
         <v>3.5</v>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>UTC+3:30</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
-      <c r="D56" t="n">
+      <c r="D57" t="n">
         <v>82</v>
       </c>
-      <c r="E56" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3581,24 +3607,24 @@
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="n">
+    <row r="58">
+      <c r="A58" t="n">
         <v>4</v>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>UTC+4</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
       </c>
-      <c r="D57" t="n">
+      <c r="D58" t="n">
         <v>267</v>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3612,54 +3638,54 @@
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" t="n">
+    <row r="59">
+      <c r="A59" t="n">
         <v>4</v>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>UTC+4</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>2/2</t>
         </is>
       </c>
-      <c r="D58" t="n">
-        <v>228</v>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="D59" t="n">
+        <v>242</v>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+4
 🇦🇲 Երևան (Yerevan) - Հայաստան (Armenia)
-🇦🇪 أبو ظبي (Abu Dhabi) - الإمارات العربية المتحدة (UAE)
+🇦🇪 أبو ظبي (Abu Dhabi) / دبي (Dubai) - الإمارات العربية المتحدة (UAE)
 🇴🇲 مَسْقَط (Muscat) - عُمان (Oman)
 🇬🇪 თბილისი (Tbilisi) - საქართველო (Georgia)
 (2/2)</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="n">
+    <row r="60">
+      <c r="A60" t="n">
         <v>4.5</v>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>UTC+4:30</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
-      <c r="D59" t="n">
+      <c r="D60" t="n">
         <v>91</v>
       </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3668,24 +3694,24 @@
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" t="n">
+    <row r="61">
+      <c r="A61" t="n">
         <v>5</v>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>UTC+5</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>1/3</t>
         </is>
       </c>
-      <c r="D60" t="n">
+      <c r="D61" t="n">
         <v>263</v>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3697,24 +3723,24 @@
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" t="n">
+    <row r="62">
+      <c r="A62" t="n">
         <v>5</v>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>UTC+5</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>2/3</t>
         </is>
       </c>
-      <c r="D61" t="n">
-        <v>260</v>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="D62" t="n">
+        <v>213</v>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3722,83 +3748,83 @@
 🇷🇺 Екатеринбург (Yekaterinburg) - Россия (Russia)
 🇹🇯 Душанбе (Dushanbe) - Тоҷикистон (Tajikistan)
 🇰🇿 Астана / Алматы (Astana / Almaty) - Қазақстан (Kazakhstan)
-🇵🇰 اسلام آباد (Islamabad) - پاکستان (Pakistan)
 (2/3)</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="n">
+    <row r="63">
+      <c r="A63" t="n">
         <v>5</v>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>UTC+5</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="D62" t="n">
-        <v>94</v>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
+      <c r="D63" t="n">
+        <v>159</v>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+5
+🇵🇰 اسلام آباد (Islamabad) / کراچی (Karachi) - پاکستان (Pakistan)
 🇲🇻 မާލެ (Malé) - ދިވެހިރާއްޖެ (Maldives)
 (3/3)</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>UTC+5:30</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>1/1</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>170</v>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
-🎇🥂🌟🪅💫💙🎉✨🍾🎆
-UTC+5:30
-🇮🇳 नई दिल्ली (New Delhi) - भारत (India)
-🇱🇰 ශ්‍රီ ජයවර්ධනපුර කෝට්ටེ་ (Sri Jayawardenepura Kotte) - ශ්‍රီ ලංකා (Sri Lanka)</t>
-        </is>
-      </c>
-    </row>
     <row r="64">
       <c r="A64" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>UTC+5:30</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>210</v>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
+🎇🥂🌟🪅💫💙🎉✨🍾🎆
+UTC+5:30
+🇮🇳 नई दिल्ली (New Delhi) / मुंबई (Mumbai) / बेंगलुरु (Bangalore) - भारत (India)
+🇱🇰 ශ්‍රီ ජයවර්ධනපුර කෝට්ටེ་ (Sri Jayawardenepura Kotte) - ශ්‍රီ ලංකා (Sri Lanka)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
         <v>5.75</v>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>UTC+5:45</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
-      <c r="D64" t="n">
+      <c r="D65" t="n">
         <v>89</v>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3807,24 +3833,24 @@
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="n">
+    <row r="66">
+      <c r="A66" t="n">
         <v>6</v>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>UTC+6</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
-      <c r="D65" t="n">
+      <c r="D66" t="n">
         <v>262</v>
       </c>
-      <c r="E65" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3837,24 +3863,24 @@
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" t="n">
+    <row r="67">
+      <c r="A67" t="n">
         <v>6.5</v>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>UTC+6:30</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
-      <c r="D66" t="n">
+      <c r="D67" t="n">
         <v>151</v>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3864,24 +3890,24 @@
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="n">
+    <row r="68">
+      <c r="A68" t="n">
         <v>7</v>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>UTC+7</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>1/3</t>
         </is>
       </c>
-      <c r="D67" t="n">
-        <v>252</v>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="D68" t="n">
+        <v>213</v>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3889,38 +3915,7 @@
 🇦🇶 Davis Station - Antarctica / Australia (Antarctica / Australia)
 🇨🇽 Flying Fish Cove - Christmas Island (Christmas Island)
 🇮🇩 Jakarta - Indonesia (Indonesia)
-🇻🇳 Hà Nội (Hanoi) - Việt Nam (Vietnam)
 (1/3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="n">
-        <v>7</v>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>UTC+7</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>2/3</t>
-        </is>
-      </c>
-      <c r="D68" t="n">
-        <v>251</v>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
-🎇🥂🌟🪅💫💙🎉✨🍾🎆
-UTC+7
-🇲🇳 Ховд (Hovd) - Монгол Улс (Mongolia)
-🇷🇺 Красноярск / Новосибирск (Krasnoyarsk / Novosibirsk) - Россия (Russia)
-🇹🇭 กรุงเทพมหานคร (Bangkok) - ประเทศไทย (Thailand)
-🇱🇦 ວຽງຈັນ (Vientiane) - ລາວ (Laos)
-(2/3)</t>
         </is>
       </c>
     </row>
@@ -3935,40 +3930,71 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
+          <t>2/3</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>248</v>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
+🎇🥂🌟🪅💫💙🎉✨🍾🎆
+UTC+7
+🇻🇳 Hà Nội (Hanoi) / Thành phố Hồ Chí Minh (Ho Chi Minh City) - Việt Nam (Vietnam)
+🇲🇳 Ховд (Hovd) - Монгол Улс (Mongolia)
+🇷🇺 Красноярск / Новосибирск (Krasnoyarsk / Novosibirsk) - Россия (Russia)
+(2/3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>7</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>UTC+7</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="D69" t="n">
-        <v>98</v>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="D70" t="n">
+        <v>183</v>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+7
+🇹🇭 กรุงเทพมหานคร (Bangkok) - ประเทศไทย (Thailand)
+🇱🇦 ວຽງຈັນ (Vientiane) - ລາວ (Laos)
 🇰🇭 ភ្នំពេញ (Phnom Penh) - កម្ពុជា (Cambodia)
 (3/3)</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" t="n">
+    <row r="71">
+      <c r="A71" t="n">
         <v>8</v>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>UTC+8</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>1/3</t>
         </is>
       </c>
-      <c r="D70" t="n">
+      <c r="D71" t="n">
         <v>224</v>
       </c>
-      <c r="E70" s="2" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -3981,24 +4007,24 @@
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" t="n">
+    <row r="72">
+      <c r="A72" t="n">
         <v>8</v>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B72" t="inlineStr">
         <is>
           <t>UTC+8</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>2/3</t>
         </is>
       </c>
-      <c r="D71" t="n">
+      <c r="D72" t="n">
         <v>264</v>
       </c>
-      <c r="E71" s="2" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4010,30 +4036,30 @@
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" t="n">
+    <row r="73">
+      <c r="A73" t="n">
         <v>8</v>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>UTC+8</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="D72" t="n">
-        <v>213</v>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
+      <c r="D73" t="n">
+        <v>228</v>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+8
 🇷🇺 Иркутск (Irkutsk) - Россия (Russia)
-🇨🇳 上海 (Shanghai) - 中国 (China)
+🇨🇳 北京 (Beijing) / 上海 (Shanghai) - 中国 (China)
 🇹🇼 台北 (Taipei) - 台灣 (Taiwan)
 🇲🇴 澳門 (Macau) - 澳門 (Macau)
 🇭🇰 香港 (Hong Kong) - 香港 (Hong Kong)
@@ -4041,24 +4067,24 @@
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" t="n">
+    <row r="74">
+      <c r="A74" t="n">
         <v>9</v>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>UTC+9</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
       </c>
-      <c r="D73" t="n">
-        <v>235</v>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="D74" t="n">
+        <v>248</v>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4067,57 +4093,57 @@
 🇮🇩 Jayapura - Indonesia (Indonesia)
 🇹🇱 Dili - Timor-Leste (Timor-Leste)
 🇷🇺 Якутск (Yakutsk) - Россия (Russia)
-🇰🇷 서울 (Seoul) - 대한민국 (South Korea)
+🇰🇷 서울 (Seoul) / 부산 (Busan) - 대한민국 (South Korea)
 (1/2)</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="n">
+    <row r="75">
+      <c r="A75" t="n">
         <v>9</v>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>UTC+9</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>2/2</t>
         </is>
       </c>
-      <c r="D74" t="n">
-        <v>126</v>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="D75" t="n">
+        <v>139</v>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
 UTC+9
 🇰🇵 평양 (Pyongyang) - 조선민주주의인민공화국 (North Korea)
-🇯🇵 東京 (Tokyo) - 日本 (Japan)
+🇯🇵 東京 (Tokyo) / 大阪 (Osaka) - 日本 (Japan)
 (2/2)</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="n">
+    <row r="76">
+      <c r="A76" t="n">
         <v>9.5</v>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>UTC+9:30</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
-      <c r="D75" t="n">
+      <c r="D76" t="n">
         <v>90</v>
       </c>
-      <c r="E75" s="2" t="inlineStr">
+      <c r="E76" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4126,24 +4152,24 @@
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="n">
+    <row r="77">
+      <c r="A77" t="n">
         <v>10</v>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>UTC+10</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
       </c>
-      <c r="D76" t="n">
+      <c r="D77" t="n">
         <v>265</v>
       </c>
-      <c r="E76" s="2" t="inlineStr">
+      <c r="E77" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4157,24 +4183,24 @@
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="n">
+    <row r="78">
+      <c r="A78" t="n">
         <v>10</v>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>UTC+10</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>2/2</t>
         </is>
       </c>
-      <c r="D77" t="n">
+      <c r="D78" t="n">
         <v>182</v>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E78" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4185,24 +4211,24 @@
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" t="n">
+    <row r="79">
+      <c r="A79" t="n">
         <v>10.5</v>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>UTC+10:30</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
-      <c r="D78" t="n">
+      <c r="D79" t="n">
         <v>86</v>
       </c>
-      <c r="E78" s="2" t="inlineStr">
+      <c r="E79" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4211,24 +4237,24 @@
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" t="n">
+    <row r="80">
+      <c r="A80" t="n">
         <v>11</v>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>UTC+11</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
       </c>
-      <c r="D79" t="n">
+      <c r="D80" t="n">
         <v>271</v>
       </c>
-      <c r="E79" s="2" t="inlineStr">
+      <c r="E80" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4242,24 +4268,24 @@
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" t="n">
+    <row r="81">
+      <c r="A81" t="n">
         <v>11</v>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>UTC+11</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>2/2</t>
         </is>
       </c>
-      <c r="D80" t="n">
+      <c r="D81" t="n">
         <v>227</v>
       </c>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E81" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4272,24 +4298,24 @@
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="n">
+    <row r="82">
+      <c r="A82" t="n">
         <v>12</v>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>UTC+12</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>1/3</t>
         </is>
       </c>
-      <c r="D81" t="n">
+      <c r="D82" t="n">
         <v>263</v>
       </c>
-      <c r="E81" s="2" t="inlineStr">
+      <c r="E82" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4303,24 +4329,24 @@
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" t="n">
+    <row r="83">
+      <c r="A83" t="n">
         <v>12</v>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>UTC+12</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>2/3</t>
         </is>
       </c>
-      <c r="D82" t="n">
+      <c r="D83" t="n">
         <v>221</v>
       </c>
-      <c r="E82" s="2" t="inlineStr">
+      <c r="E83" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4334,24 +4360,24 @@
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" t="n">
+    <row r="84">
+      <c r="A84" t="n">
         <v>12</v>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>UTC+12</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="D83" t="n">
+      <c r="D84" t="n">
         <v>112</v>
       </c>
-      <c r="E83" s="2" t="inlineStr">
+      <c r="E84" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4361,24 +4387,24 @@
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" t="n">
+    <row r="85">
+      <c r="A85" t="n">
         <v>13</v>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>UTC+13</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
       </c>
-      <c r="D84" t="n">
+      <c r="D85" t="n">
         <v>195</v>
       </c>
-      <c r="E84" s="2" t="inlineStr">
+      <c r="E85" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4389,24 +4415,24 @@
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="n">
+    <row r="86">
+      <c r="A86" t="n">
         <v>13</v>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>UTC+13</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>2/2</t>
         </is>
       </c>
-      <c r="D85" t="n">
+      <c r="D86" t="n">
         <v>230</v>
       </c>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="E86" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4419,24 +4445,24 @@
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="n">
+    <row r="87">
+      <c r="A87" t="n">
         <v>13.75</v>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>UTC+13:45</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
-      <c r="D86" t="n">
+      <c r="D87" t="n">
         <v>103</v>
       </c>
-      <c r="E86" s="2" t="inlineStr">
+      <c r="E87" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆
@@ -4445,24 +4471,24 @@
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="n">
+    <row r="88">
+      <c r="A88" t="n">
         <v>14</v>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>UTC+14</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
-      <c r="D87" t="n">
+      <c r="D88" t="n">
         <v>139</v>
       </c>
-      <c r="E87" s="2" t="inlineStr">
+      <c r="E88" s="2" t="inlineStr">
         <is>
           <t>2️⃣0️⃣ #HappyNewYear 2️⃣7️⃣
 🎇🥂🌟🪅💫💙🎉✨🍾🎆

</xml_diff>